<commit_message>
PAUSED (task182, task190, task193, task194, task195): checkpoint, five builds mid-pass
Checkpoint only, no status change. task182 has a zip and a submission and is closing
on its stage-3 gates, task190 is re-cutting the goldens, asks and documents onto the
nearest-fifty basis on the mass-balance reading, task193 is waiting on stage-4 work
of its own after redistributing its pins, and task194 and task195 are on their fix
passes. task192's repair pass is briefed and running.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task190/golden/structured_cash_deposits_2027.xlsx
+++ b/task190/golden/structured_cash_deposits_2027.xlsx
@@ -37,7 +37,7 @@
     <t>Largest segment</t>
   </si>
   <si>
-    <t>Transport and courier, 90</t>
+    <t>Transport and courier, 150</t>
   </si>
   <si>
     <t>Business segment</t>
@@ -49,22 +49,22 @@
     <t>Transport and courier</t>
   </si>
   <si>
+    <t>Grocery and convenience</t>
+  </si>
+  <si>
+    <t>Fuel and automotive</t>
+  </si>
+  <si>
+    <t>Hospitality</t>
+  </si>
+  <si>
+    <t>Personal services</t>
+  </si>
+  <si>
     <t>Trades and construction</t>
   </si>
   <si>
-    <t>Grocery and convenience</t>
-  </si>
-  <si>
-    <t>Hospitality</t>
-  </si>
-  <si>
     <t>Clubs and community</t>
-  </si>
-  <si>
-    <t>Fuel and automotive</t>
-  </si>
-  <si>
-    <t>Personal services</t>
   </si>
   <si>
     <t>Rural supply and horticulture</t>
@@ -512,7 +512,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -539,10 +539,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="7">
-        <v>2300</v>
+        <v>10433</v>
       </c>
       <c r="C8" s="7">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -550,10 +550,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="7">
-        <v>3684</v>
+        <v>15131</v>
       </c>
       <c r="C9" s="7">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -561,10 +561,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="7">
-        <v>14111</v>
+        <v>4175</v>
       </c>
       <c r="C10" s="7">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -572,10 +572,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="7">
-        <v>11297</v>
+        <v>4758</v>
       </c>
       <c r="C11" s="7">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -583,10 +583,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="7">
-        <v>1836</v>
+        <v>3993</v>
       </c>
       <c r="C12" s="7">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -594,10 +594,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="7">
-        <v>6658</v>
+        <v>3168</v>
       </c>
       <c r="C13" s="7">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -605,10 +605,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="7">
-        <v>2036</v>
+        <v>2718</v>
       </c>
       <c r="C14" s="7">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -616,10 +616,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="7">
-        <v>3042</v>
+        <v>2396</v>
       </c>
       <c r="C15" s="7">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -627,10 +627,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="9">
-        <v>44964</v>
+        <v>46772</v>
       </c>
       <c r="C16" s="9">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>